<commit_message>
Deploying to gh-pages from @ insysbio/faah-inhibitor@e608bdb02c82afba8067ad4e0f4a52be52a0dc58 🚀
</commit_message>
<xml_diff>
--- a/table/output.heta.xlsx
+++ b/table/output.heta.xlsx
@@ -490,13 +490,13 @@
         <v>0.10.0</v>
       </c>
       <c r="Q2" t="str">
-        <v>2026-03-19T15:46:09.034Z</v>
+        <v>2026-03-19T17:48:11.232Z</v>
       </c>
       <c r="R2" t="str">
         <v>faah-inhibitor</v>
       </c>
       <c r="S2" t="str">
-        <v>1.0.2</v>
+        <v>1.0.3</v>
       </c>
       <c r="T2" t="str">
         <v>Table</v>

</xml_diff>